<commit_message>
Aggiunti Matteo Ceccaglia e Daniela Valli in Prova_Github.xlsx
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017fiaA1CJzDW9MvYbP9S6M1
</commit_message>
<xml_diff>
--- a/Prova_Github.xlsx
+++ b/Prova_Github.xlsx
@@ -1,68 +1,33 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
-  <workbookPr defaultThemeVersion="202300"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\matteo.ceccaglia\Desktop\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{2AFDCF1C-BE35-4CCD-9741-7E2C2A68D919}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <workbookPr/>
   <bookViews>
-    <workbookView xWindow="22932" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{63FF4837-E065-462C-A0E9-512192044237}"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="22932" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Foglio1" sheetId="1" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Foglio1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029"/>
-  <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
-      <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
-      <xlwcv:version setVersion="2"/>
-    </ext>
-  </extLst>
+  <definedNames/>
+  <calcPr calcId="191029" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2" uniqueCount="2">
-  <si>
-    <t>Cognome</t>
-  </si>
-  <si>
-    <t>Nome</t>
-  </si>
-</sst>
-</file>
-
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="0"/>
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
+      <color theme="1"/>
+      <sz val="11"/>
       <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
     <fill>
-      <patternFill patternType="none"/>
+      <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -81,21 +46,80 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normale" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
 </file>
 
@@ -415,16 +439,48 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7D9AC052-1D8B-4900-A519-1FEE7F8C9DA4}">
-  <dimension ref="A1:B1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
-        <v>1</v>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Cognome</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Nome</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Ceccaglia</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Matteo</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Valli</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Daniela</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Aggiunti Lorenzo Montali e Cristiano Paci in Prova_Github.xlsx
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017fiaA1CJzDW9MvYbP9S6M1
</commit_message>
<xml_diff>
--- a/Prova_Github.xlsx
+++ b/Prova_Github.xlsx
@@ -444,7 +444,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B3"/>
+  <dimension ref="A1:B5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -480,6 +480,30 @@
       <c r="B3" t="inlineStr">
         <is>
           <t>Daniela</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Montali</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Lorenzo</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Paci</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Cristiano</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Aggiunti Michael Casali e Federica De silvestri in Prova_Github.xlsx
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017fiaA1CJzDW9MvYbP9S6M1
</commit_message>
<xml_diff>
--- a/Prova_Github.xlsx
+++ b/Prova_Github.xlsx
@@ -444,7 +444,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B5"/>
+  <dimension ref="A1:B7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -507,6 +507,30 @@
         </is>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Casali</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Michael</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>De silvestri</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Federica</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>